<commit_message>
Record public static demo acceptance and client walkthrough
</commit_message>
<xml_diff>
--- a/development/evidence/client-demo/emerald-DEMO-activity-2026-10-21-2026-10-21.xlsx
+++ b/development/evidence/client-demo/emerald-DEMO-activity-2026-10-21-2026-10-21.xlsx
@@ -67,7 +67,7 @@
     <t>Al Quoz</t>
   </si>
   <si>
-    <t>21/10/2026, 07:25</t>
+    <t>21/10/2026, 07:37</t>
   </si>
   <si>
     <t>Follow-up Required</t>
@@ -76,10 +76,10 @@
     <t>Fictional client demo discussion — മാതൃക — نموذج</t>
   </si>
   <si>
-    <t>21/10/2026, 07:23</t>
-  </si>
-  <si>
-    <t>21/10/2026, 07:24</t>
+    <t>21/10/2026, 07:35</t>
+  </si>
+  <si>
+    <t>21/10/2026, 07:36</t>
   </si>
   <si>
     <t>Regular Visit</t>

</xml_diff>